<commit_message>
feat: release final v0.22.0 - soporte jerarquias 4E, minutas estructuradas, voz y dashboard
</commit_message>
<xml_diff>
--- a/releases/plantilla_excel_v1_1/plantilla_plan_trabajo_jira_v1_1.xlsx
+++ b/releases/plantilla_excel_v1_1/plantilla_plan_trabajo_jira_v1_1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLAN_DE_TRABAJO" sheetId="1" r:id="Rb8bb7ed1471d427e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYUDA" sheetId="2" r:id="R80611b1b48f74519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJEMPLO_MIGRADO" sheetId="3" r:id="R0713e6258c7d4a9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLAN_DE_TRABAJO" sheetId="1" r:id="R3e653ee35ead4654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AYUDA" sheetId="2" r:id="Rd7ab9d359dd94f53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJEMPLO_MIGRADO" sheetId="3" r:id="R24db39e8d8db4893"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -371,12 +371,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlanTrabajoTable" displayName="PlanTrabajoTable" ref="A5:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PlanTrabajoTable" displayName="PlanTrabajoTable" ref="A5:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G55"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Actividad *"/>
     <x:tableColumn id="2" name="Responsable *"/>
-    <x:tableColumn id="3" name="Grupo_o_Modulo"/>
+    <x:tableColumn id="3" name="Frente_de_trabajo_o_Proyecto"/>
     <x:tableColumn id="4" name="Contexto_o_Resultado"/>
     <x:tableColumn id="5" name="Fecha_Objetivo"/>
     <x:tableColumn id="6" name="Estado_Actual"/>
@@ -387,11 +387,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="EjemploMigradoTable" displayName="EjemploMigradoTable" ref="A5:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EjemploMigradoTable" displayName="EjemploMigradoTable" ref="A5:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:J17"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Actividad"/>
     <x:tableColumn id="2" name="Responsable"/>
-    <x:tableColumn id="3" name="Grupo_o_Modulo"/>
+    <x:tableColumn id="3" name="Frente_de_trabajo_o_Proyecto"/>
     <x:tableColumn id="4" name="Contexto_o_Resultado"/>
     <x:tableColumn id="5" name="Fecha_Objetivo"/>
     <x:tableColumn id="6" name="Estado_Actual"/>
@@ -1277,7 +1278,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72d1b288167c43ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd594dab984814e32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2143,7 +2144,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf90575d3cb4ad6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac879fc38894550"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>